<commit_message>
feat: add emitter or receiver role to the transceiver
starting from now, only receiver can compute penalties or rx_power

Signed-off-by: JennyLescop <jenny.lescop@orange.com>
Change-Id: I3a9cdc19643c353eb589440a856097ea27e99ff5
</commit_message>
<xml_diff>
--- a/tests/data/testTopology_PATH_expected.xlsx
+++ b/tests/data/testTopology_PATH_expected.xlsx
@@ -388,9 +388,6 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.0 ms
 	- Actual pch out:: 0.00 dBm
-	- CD penalty: None dB
-	- PMD penalty:: None dB
-	- PDL penalty:: None dB
 </t>
         </is>
       </c>
@@ -510,9 +507,6 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.0 ms
 	- Actual pch out:: 0.00 dBm
-	- CD penalty: None dB
-	- PMD penalty:: None dB
-	- PDL penalty:: None dB
 </t>
         </is>
       </c>
@@ -797,9 +791,6 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.0 ms
 	- Actual pch out:: 0.00 dBm
-	- CD penalty: None dB
-	- PMD penalty:: None dB
-	- PDL penalty:: None dB
 </t>
         </is>
       </c>
@@ -948,9 +939,6 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.0 ms
 	- Actual pch out:: 0.00 dBm
-	- CD penalty: None dB
-	- PMD penalty:: None dB
-	- PDL penalty:: None dB
 </t>
         </is>
       </c>
@@ -1243,9 +1231,6 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.0 ms
 	- Actual pch out:: 0.00 dBm
-	- CD penalty: None dB
-	- PMD penalty:: None dB
-	- PDL penalty:: None dB
 </t>
         </is>
       </c>

</xml_diff>